<commit_message>
Update as_building drawing v1.16 spartak
Закончил стены в библиотеке
</commit_message>
<xml_diff>
--- a/vor_spartac.xlsx
+++ b/vor_spartac.xlsx
@@ -4,19 +4,19 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="23265" yWindow="5565" windowWidth="5535" windowHeight="6105" activeTab="1"/>
+    <workbookView xWindow="23265" yWindow="5565" windowWidth="5535" windowHeight="6105" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Пример" sheetId="1" r:id="rId1"/>
     <sheet name="Лист2" sheetId="2" r:id="rId2"/>
-    <sheet name="Лист3" sheetId="3" r:id="rId3"/>
+    <sheet name="библиотека" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="48">
   <si>
     <t>Штукатурка цементным составом толщиной 16‐20 мм</t>
   </si>
@@ -154,13 +154,19 @@
   </si>
   <si>
     <t>332 п.м</t>
+  </si>
+  <si>
+    <t>14.80 п.м.</t>
+  </si>
+  <si>
+    <t>698.56 п.м.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,6 +185,21 @@
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="ГОСТ тип А"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="ГОСТ тип А"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="ГОСТ тип А"/>
       <family val="2"/>
@@ -287,7 +308,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -392,6 +413,59 @@
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1685,9 +1759,231 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A15:E33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="13.7109375" style="37" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="55"/>
+    <col min="3" max="3" width="59.5703125" style="37" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" style="55" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" style="37" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="37"/>
+  </cols>
+  <sheetData>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="38"/>
+      <c r="B15" s="39"/>
+      <c r="C15" s="40" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="41"/>
+      <c r="E15" s="42"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="38"/>
+      <c r="B16" s="43" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="44" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="46" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="38"/>
+      <c r="B17" s="43">
+        <v>1</v>
+      </c>
+      <c r="C17" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="45">
+        <v>1035.18</v>
+      </c>
+      <c r="E17" s="46"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="38"/>
+      <c r="B18" s="43">
+        <v>2</v>
+      </c>
+      <c r="C18" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="45">
+        <v>66.28</v>
+      </c>
+      <c r="E18" s="46"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="38"/>
+      <c r="B19" s="43">
+        <v>3</v>
+      </c>
+      <c r="C19" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" s="45">
+        <f>D17</f>
+        <v>1035.18</v>
+      </c>
+      <c r="E19" s="46"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="38"/>
+      <c r="B20" s="43">
+        <v>4</v>
+      </c>
+      <c r="C20" s="44" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="45">
+        <f>D18</f>
+        <v>66.28</v>
+      </c>
+      <c r="E20" s="46"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="38"/>
+      <c r="B21" s="43">
+        <v>5</v>
+      </c>
+      <c r="C21" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" s="45" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" s="46"/>
+    </row>
+    <row r="22" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="38"/>
+      <c r="B22" s="43">
+        <v>6</v>
+      </c>
+      <c r="C22" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="D22" s="45">
+        <f>1282+128</f>
+        <v>1410</v>
+      </c>
+      <c r="E22" s="46"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="38"/>
+      <c r="B23" s="48">
+        <v>6.1</v>
+      </c>
+      <c r="C23" s="44" t="s">
+        <v>33</v>
+      </c>
+      <c r="D23" s="45"/>
+      <c r="E23" s="46">
+        <f>D22*0.15</f>
+        <v>211.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="38"/>
+      <c r="B24" s="48">
+        <v>6.2</v>
+      </c>
+      <c r="C24" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="45"/>
+      <c r="E24" s="46">
+        <f>D22*0.3</f>
+        <v>423</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="38" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="39"/>
+      <c r="C26" s="49" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="50"/>
+      <c r="E26" s="51"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="38"/>
+      <c r="B27" s="43" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="44" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="45" t="s">
+        <v>29</v>
+      </c>
+      <c r="E27" s="51"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="38"/>
+      <c r="B28" s="43">
+        <v>1</v>
+      </c>
+      <c r="C28" s="44" t="s">
+        <v>0</v>
+      </c>
+      <c r="D28" s="45">
+        <v>19.059999999999999</v>
+      </c>
+      <c r="E28" s="51"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="38"/>
+      <c r="B29" s="43">
+        <v>2</v>
+      </c>
+      <c r="C29" s="52" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="45" t="s">
+        <v>46</v>
+      </c>
+      <c r="E29" s="51"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="54"/>
+      <c r="C31" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" s="54"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B32" s="54" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="53" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" s="54" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B33" s="54">
+        <v>1</v>
+      </c>
+      <c r="C33" s="53" t="s">
+        <v>38</v>
+      </c>
+      <c r="D33" s="54">
+        <v>25.85</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>